<commit_message>
Accept productOrder source file aliases
</commit_message>
<xml_diff>
--- a/src/main/resources/lia-report-spec.xlsx
+++ b/src/main/resources/lia-report-spec.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/linjiaying/IdeaProjects/LIA-batch/src/main/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EF592DC-C8BA-894D-BEEE-CEB08EFCD0A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E7E43C0-2671-BD45-AE2D-624FB15D4C27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="580" yWindow="660" windowWidth="28240" windowHeight="17240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="580" yWindow="660" windowWidth="28240" windowHeight="17240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="outputFileDetail" sheetId="1" r:id="rId1"/>
@@ -170,9 +170,6 @@
     <t>商品代號</t>
   </si>
   <si>
-    <t>productOrder</t>
-  </si>
-  <si>
     <t>productOrderNo</t>
   </si>
   <si>
@@ -182,6 +179,10 @@
     <t>choose
 (1:selectReportData()
 (2:selectProductOrderReportData()</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>product_Order</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1060,10 +1061,10 @@
         <v>0</v>
       </c>
       <c r="J12" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K12" s="6" t="s">
         <v>49</v>
-      </c>
-      <c r="K12" s="6" t="s">
-        <v>50</v>
       </c>
       <c r="M12" t="s">
         <v>26</v>
@@ -1086,7 +1087,7 @@
         <v>29</v>
       </c>
       <c r="F13">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="G13">
         <v>20</v>
@@ -1095,10 +1096,10 @@
         <v>24</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="M13" t="s">
         <v>26</v>
@@ -1129,7 +1130,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>1</v>

</xml_diff>